<commit_message>
fix bug in 15th excel file Magni
</commit_message>
<xml_diff>
--- a/Dingli/JCPT0808-1614 Магни  备件手册  英文（SM0117217_Rev1.0）_модели.xlsx
+++ b/Dingli/JCPT0808-1614 Магни  备件手册  英文（SM0117217_Rev1.0）_модели.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Parts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,37 +417,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Part Number</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Node</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Models</t>
         </is>
@@ -492,7 +480,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -554,7 +542,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -585,7 +573,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -616,7 +604,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -647,7 +635,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -678,7 +666,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -709,7 +697,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -740,7 +728,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -771,7 +759,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -864,7 +852,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -895,7 +883,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -926,7 +914,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1009,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1040,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1071,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1102,7 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1226,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1381,7 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1412,7 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1443,7 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1474,7 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1505,7 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1536,7 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1567,7 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1598,7 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1629,7 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1660,7 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1691,7 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1722,7 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1753,7 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1784,7 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1815,7 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1846,7 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1877,7 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1908,7 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1939,7 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1970,7 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2065,7 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2096,7 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2127,7 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2190,7 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2221,7 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2283,7 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2314,7 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2345,7 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2376,7 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2407,7 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2438,7 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2469,7 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2500,7 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2531,7 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2562,7 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2593,7 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2624,7 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2667,7 +2655,7 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2686,7 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2717,7 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2748,7 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2779,7 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2811,7 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2843,7 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2968,7 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3030,7 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3061,7 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3092,7 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3123,7 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3154,7 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3216,7 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3247,7 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3322,7 +3310,7 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3341,7 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3415,7 +3403,7 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3434,7 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3465,7 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3508,7 +3496,7 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3539,7 +3527,7 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3558,7 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3589,7 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3620,7 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3652,7 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3683,7 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3714,7 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3745,7 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3788,7 +3776,7 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3819,7 +3807,7 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3850,7 +3838,7 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3943,7 +3931,7 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3962,7 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4005,7 +3993,7 @@
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4024,7 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4055,7 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4086,7 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4149,7 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4192,7 +4180,7 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4211,7 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4242,7 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4285,7 +4273,7 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4368,7 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4399,7 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4442,7 +4430,7 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4473,7 +4461,7 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4492,7 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4523,7 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4585,7 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4616,7 @@
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4659,7 +4647,7 @@
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4678,7 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4709,7 @@
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4846,7 +4834,7 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4865,7 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4896,7 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4939,7 +4927,7 @@
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4958,7 @@
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5001,7 +4989,7 @@
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5082,7 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5113,7 @@
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5271,7 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5314,7 +5302,7 @@
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5364,7 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5395,7 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5426,7 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5457,7 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5488,7 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5531,7 +5519,7 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5562,7 +5550,7 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5593,7 +5581,7 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5624,7 +5612,7 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5643,7 @@
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5686,7 +5674,7 @@
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5705,7 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -5779,7 +5767,7 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6419,7 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7516,7 +7504,7 @@
       <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7578,7 +7566,7 @@
       <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7609,7 +7597,7 @@
       <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7628,7 @@
       <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7702,7 +7690,7 @@
       <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7857,7 +7845,7 @@
       <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7888,7 +7876,7 @@
       <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7919,7 +7907,7 @@
       <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7950,7 +7938,7 @@
       <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -7983,7 +7971,7 @@
       <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8002,7 @@
       <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -8169,7 +8157,7 @@
       <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -8200,7 +8188,7 @@
       <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -8231,7 +8219,7 @@
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8904,7 @@
       <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -8978,7 +8966,7 @@
       <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9009,7 +8997,7 @@
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9040,7 +9028,7 @@
       <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9071,7 +9059,7 @@
       <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9102,7 +9090,7 @@
       <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9133,7 +9121,7 @@
       <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9164,7 +9152,7 @@
       <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9226,7 +9214,7 @@
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9320,7 +9308,7 @@
       <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9432,7 @@
       <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9475,7 +9463,7 @@
       <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9506,7 +9494,7 @@
       <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9537,7 +9525,7 @@
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9568,7 +9556,7 @@
       <c r="F294" t="inlineStr"/>
       <c r="G294" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9599,7 +9587,7 @@
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9630,7 +9618,7 @@
       <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9661,7 +9649,7 @@
       <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9692,7 +9680,7 @@
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9723,7 +9711,7 @@
       <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9754,7 +9742,7 @@
       <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9785,7 +9773,7 @@
       <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9816,7 +9804,7 @@
       <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9847,7 +9835,7 @@
       <c r="F303" t="inlineStr"/>
       <c r="G303" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9878,7 +9866,7 @@
       <c r="F304" t="inlineStr"/>
       <c r="G304" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9909,7 +9897,7 @@
       <c r="F305" t="inlineStr"/>
       <c r="G305" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9940,7 +9928,7 @@
       <c r="F306" t="inlineStr"/>
       <c r="G306" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -9971,7 +9959,7 @@
       <c r="F307" t="inlineStr"/>
       <c r="G307" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10002,7 +9990,7 @@
       <c r="F308" t="inlineStr"/>
       <c r="G308" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10033,7 +10021,7 @@
       <c r="F309" t="inlineStr"/>
       <c r="G309" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10064,7 +10052,7 @@
       <c r="F310" t="inlineStr"/>
       <c r="G310" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10095,7 +10083,7 @@
       <c r="F311" t="inlineStr"/>
       <c r="G311" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10126,7 +10114,7 @@
       <c r="F312" t="inlineStr"/>
       <c r="G312" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10157,7 +10145,7 @@
       <c r="F313" t="inlineStr"/>
       <c r="G313" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10250,7 +10238,7 @@
       <c r="F316" t="inlineStr"/>
       <c r="G316" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10344,7 +10332,7 @@
       <c r="F319" t="inlineStr"/>
       <c r="G319" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10375,7 +10363,7 @@
       <c r="F320" t="inlineStr"/>
       <c r="G320" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10406,7 +10394,7 @@
       <c r="F321" t="inlineStr"/>
       <c r="G321" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10437,7 +10425,7 @@
       <c r="F322" t="inlineStr"/>
       <c r="G322" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10468,7 +10456,7 @@
       <c r="F323" t="inlineStr"/>
       <c r="G323" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10499,7 +10487,7 @@
       <c r="F324" t="inlineStr"/>
       <c r="G324" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10530,7 +10518,7 @@
       <c r="F325" t="inlineStr"/>
       <c r="G325" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10561,7 +10549,7 @@
       <c r="F326" t="inlineStr"/>
       <c r="G326" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10592,7 +10580,7 @@
       <c r="F327" t="inlineStr"/>
       <c r="G327" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10623,7 +10611,7 @@
       <c r="F328" t="inlineStr"/>
       <c r="G328" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10654,7 +10642,7 @@
       <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10685,7 +10673,7 @@
       <c r="F330" t="inlineStr"/>
       <c r="G330" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10716,7 +10704,7 @@
       <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10747,7 +10735,7 @@
       <c r="F332" t="inlineStr"/>
       <c r="G332" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10778,7 +10766,7 @@
       <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10809,7 +10797,7 @@
       <c r="F334" t="inlineStr"/>
       <c r="G334" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10840,7 +10828,7 @@
       <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10871,7 +10859,7 @@
       <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10890,7 @@
       <c r="F337" t="inlineStr"/>
       <c r="G337" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10933,7 +10921,7 @@
       <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10964,7 +10952,7 @@
       <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -10995,7 +10983,7 @@
       <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11026,7 +11014,7 @@
       <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11368,7 +11356,7 @@
       <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11399,7 +11387,7 @@
       <c r="F353" t="inlineStr"/>
       <c r="G353" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11430,7 +11418,7 @@
       <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11461,7 +11449,7 @@
       <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11492,7 +11480,7 @@
       <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11523,7 +11511,7 @@
       <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11554,7 +11542,7 @@
       <c r="F358" t="inlineStr"/>
       <c r="G358" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11585,7 +11573,7 @@
       <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11604,7 @@
       <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -11999,7 +11987,7 @@
       <c r="F372" t="inlineStr"/>
       <c r="G372" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12031,7 +12019,7 @@
       <c r="F373" t="inlineStr"/>
       <c r="G373" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12062,7 +12050,7 @@
       <c r="F374" t="inlineStr"/>
       <c r="G374" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12093,7 +12081,7 @@
       <c r="F375" t="inlineStr"/>
       <c r="G375" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12124,7 +12112,7 @@
       <c r="F376" t="inlineStr"/>
       <c r="G376" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12155,7 +12143,7 @@
       <c r="F377" t="inlineStr"/>
       <c r="G377" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12281,7 +12269,7 @@
       <c r="F381" t="inlineStr"/>
       <c r="G381" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12379,7 +12367,7 @@
       <c r="F384" t="inlineStr"/>
       <c r="G384" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12410,7 +12398,7 @@
       <c r="F385" t="inlineStr"/>
       <c r="G385" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -12538,7 +12526,7 @@
       <c r="F389" t="inlineStr"/>
       <c r="G389" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13039,7 +13027,7 @@
       <c r="F405" t="inlineStr"/>
       <c r="G405" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13070,7 +13058,7 @@
       <c r="F406" t="inlineStr"/>
       <c r="G406" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13349,7 +13337,7 @@
       <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13380,7 +13368,7 @@
       <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13411,7 +13399,7 @@
       <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13442,7 +13430,7 @@
       <c r="F418" t="inlineStr"/>
       <c r="G418" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13535,7 +13523,7 @@
       <c r="F421" t="inlineStr"/>
       <c r="G421" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13566,7 +13554,7 @@
       <c r="F422" t="inlineStr"/>
       <c r="G422" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -13597,7 +13585,7 @@
       <c r="F423" t="inlineStr"/>
       <c r="G423" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -14590,7 +14578,7 @@
       <c r="F455" t="inlineStr"/>
       <c r="G455" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -14621,7 +14609,7 @@
       <c r="F456" t="inlineStr"/>
       <c r="G456" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -14652,7 +14640,7 @@
       <c r="F457" t="inlineStr"/>
       <c r="G457" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -14683,7 +14671,7 @@
       <c r="F458" t="inlineStr"/>
       <c r="G458" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -14714,7 +14702,7 @@
       <c r="F459" t="inlineStr"/>
       <c r="G459" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15057,7 +15045,7 @@
       <c r="F470" t="inlineStr"/>
       <c r="G470" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15150,7 +15138,7 @@
       <c r="F473" t="inlineStr"/>
       <c r="G473" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15182,7 +15170,7 @@
       <c r="F474" t="inlineStr"/>
       <c r="G474" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15213,7 +15201,7 @@
       <c r="F475" t="inlineStr"/>
       <c r="G475" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15275,7 +15263,7 @@
       <c r="F477" t="inlineStr"/>
       <c r="G477" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15369,7 +15357,7 @@
       <c r="F480" t="inlineStr"/>
       <c r="G480" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15400,7 +15388,7 @@
       <c r="F481" t="inlineStr"/>
       <c r="G481" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15431,7 +15419,7 @@
       <c r="F482" t="inlineStr"/>
       <c r="G482" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15462,7 +15450,7 @@
       <c r="F483" t="inlineStr"/>
       <c r="G483" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15493,7 +15481,7 @@
       <c r="F484" t="inlineStr"/>
       <c r="G484" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15524,7 +15512,7 @@
       <c r="F485" t="inlineStr"/>
       <c r="G485" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15555,7 +15543,7 @@
       <c r="F486" t="inlineStr"/>
       <c r="G486" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15586,7 +15574,7 @@
       <c r="F487" t="inlineStr"/>
       <c r="G487" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15617,7 +15605,7 @@
       <c r="F488" t="inlineStr"/>
       <c r="G488" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15648,7 +15636,7 @@
       <c r="F489" t="inlineStr"/>
       <c r="G489" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15679,7 +15667,7 @@
       <c r="F490" t="inlineStr"/>
       <c r="G490" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15710,7 +15698,7 @@
       <c r="F491" t="inlineStr"/>
       <c r="G491" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15741,7 +15729,7 @@
       <c r="F492" t="inlineStr"/>
       <c r="G492" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15772,7 +15760,7 @@
       <c r="F493" t="inlineStr"/>
       <c r="G493" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15803,7 +15791,7 @@
       <c r="F494" t="inlineStr"/>
       <c r="G494" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15866,7 +15854,7 @@
       <c r="F496" t="inlineStr"/>
       <c r="G496" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15897,7 +15885,7 @@
       <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15928,7 +15916,7 @@
       <c r="F498" t="inlineStr"/>
       <c r="G498" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -15959,7 +15947,7 @@
       <c r="F499" t="inlineStr"/>
       <c r="G499" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16009,7 @@
       <c r="F501" t="inlineStr"/>
       <c r="G501" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16052,7 +16040,7 @@
       <c r="F502" t="inlineStr"/>
       <c r="G502" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16083,7 +16071,7 @@
       <c r="F503" t="inlineStr"/>
       <c r="G503" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16114,7 +16102,7 @@
       <c r="F504" t="inlineStr"/>
       <c r="G504" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16145,7 +16133,7 @@
       <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16208,7 +16196,7 @@
       <c r="F507" t="inlineStr"/>
       <c r="G507" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16239,7 +16227,7 @@
       <c r="F508" t="inlineStr"/>
       <c r="G508" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16302,7 +16290,7 @@
       <c r="F510" t="inlineStr"/>
       <c r="G510" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16333,7 +16321,7 @@
       <c r="F511" t="inlineStr"/>
       <c r="G511" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16397,7 +16385,7 @@
       <c r="F513" t="inlineStr"/>
       <c r="G513" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16459,7 +16447,7 @@
       <c r="F515" t="inlineStr"/>
       <c r="G515" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16490,7 +16478,7 @@
       <c r="F516" t="inlineStr"/>
       <c r="G516" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16521,7 +16509,7 @@
       <c r="F517" t="inlineStr"/>
       <c r="G517" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16552,7 +16540,7 @@
       <c r="F518" t="inlineStr"/>
       <c r="G518" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16583,7 +16571,7 @@
       <c r="F519" t="inlineStr"/>
       <c r="G519" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16778,7 +16766,7 @@
       <c r="F525" t="inlineStr"/>
       <c r="G525" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16809,7 +16797,7 @@
       <c r="F526" t="inlineStr"/>
       <c r="G526" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16840,7 +16828,7 @@
       <c r="F527" t="inlineStr"/>
       <c r="G527" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -16964,7 +16952,7 @@
       <c r="F531" t="inlineStr"/>
       <c r="G531" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17061,7 +17049,7 @@
       <c r="F534" t="inlineStr"/>
       <c r="G534" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17092,7 +17080,7 @@
       <c r="F535" t="inlineStr"/>
       <c r="G535" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17123,7 +17111,7 @@
       <c r="F536" t="inlineStr"/>
       <c r="G536" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17187,7 +17175,7 @@
       <c r="F538" t="inlineStr"/>
       <c r="G538" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17218,7 +17206,7 @@
       <c r="F539" t="inlineStr"/>
       <c r="G539" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17249,7 +17237,7 @@
       <c r="F540" t="inlineStr"/>
       <c r="G540" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17280,7 +17268,7 @@
       <c r="F541" t="inlineStr"/>
       <c r="G541" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17311,7 +17299,7 @@
       <c r="F542" t="inlineStr"/>
       <c r="G542" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17342,7 +17330,7 @@
       <c r="F543" t="inlineStr"/>
       <c r="G543" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17373,7 +17361,7 @@
       <c r="F544" t="inlineStr"/>
       <c r="G544" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17404,7 +17392,7 @@
       <c r="F545" t="inlineStr"/>
       <c r="G545" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>
@@ -17435,7 +17423,7 @@
       <c r="F546" t="inlineStr"/>
       <c r="G546" t="inlineStr">
         <is>
-          <t>JCPT0808; JCPT0812; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
+          <t>JCPT0808; JCPT1008; JCPT1012; JCPT1212; JCPT1412; JCPT1612; JCPT1614</t>
         </is>
       </c>
     </row>

</xml_diff>